<commit_message>
Migrate to Open-Meteo API with config-driven architecture
Replace HTML scraping (Météociel) with Open-Meteo Ensemble API. Switch from individual Excel forecasts to unified Parquet database. Add support for all 4 daily cycles (0Z/6Z/12Z/18Z) with per-model cycle detection. Introduce centralized config.py for models, variables, and thresholds. Redesign dashboard to compute all statistics on-the-fly from raw members. Add cross-validation between legacy and new pipelines. Update workflow cron to 4×/day polling.
</commit_message>
<xml_diff>
--- a/Forecasts/Forecast-30062026-0Z.xlsx
+++ b/Forecasts/Forecast-30062026-0Z.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Comparaison Modèles" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Synthèse" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ECMWF" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AIFS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="GEFS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparaison Modèles" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ECMWF" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AIFS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GEFS" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -653,7 +653,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 30/06/2026 11:10</t>
+          <t>Généré le : 30/06/2026 17:30</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 30/06/2026 11:10</t>
+          <t>Généré le : 30/06/2026 17:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Metadata API for authoritative run_date detection
Implement Open-Meteo Metadata API (last_run_initialisation_time) to determine model cycle times accurately, eliminating heuristic ambiguity. Queries execute in parallel and don't count toward quota. Falls back to infer_run_date() if endpoint unavailable. Logs audit warnings when metadata and heuristic diverge by >6h.

Also:
- Refine _nearest_cron_hour() with minute-level resolution for better cron slot detection
- Parse legacy xlsx run_date from Météociel headers for cross-validation alignment
- Add _nearest_run_date() to find actual model cycles in database (not just calendar date)
</commit_message>
<xml_diff>
--- a/Forecasts/Forecast-30062026-0Z.xlsx
+++ b/Forecasts/Forecast-30062026-0Z.xlsx
@@ -653,7 +653,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 30/06/2026 17:30</t>
+          <t>Généré le : 01/07/2026 10:21</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 30/06/2026 17:30</t>
+          <t>Généré le : 01/07/2026 10:21</t>
         </is>
       </c>
     </row>

</xml_diff>